<commit_message>
Docs: the refresh runs hyperliquid_bot's array sync, not its main.py
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/quickfix_all_markets_daily.xlsx
+++ b/output/quickfix_all_markets_daily.xlsx
@@ -554,11 +554,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F2" t="n">
         <v>9</v>
@@ -602,17 +602,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -624,16 +624,16 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>100</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>13.92</v>
+        <v>16.93</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>113921.15</v>
+        <v>116929.81</v>
       </c>
     </row>
     <row r="4">
@@ -650,11 +650,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F4" t="n">
         <v>9</v>
@@ -687,7 +687,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dow_Futures_E_mini</t>
+          <t>Corn_CBOT_Futures</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -698,23 +698,23 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="n">
         <v>3</v>
       </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -723,46 +723,46 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>66.7</v>
+        <v>75</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>7.1</v>
+        <v>7.38</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>107095.5</v>
+        <v>107383.44</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Live_Cattle_Futures_CME</t>
+          <t>Dow_Futures_E_mini</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>136</v>
+        <v>65</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -771,34 +771,34 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>75</v>
+        <v>66.7</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>6.63</v>
+        <v>7.1</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>106631.02</v>
+        <v>107095.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NY_Platinum_Futures</t>
+          <t>Live_Cattle_Futures_CME</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-01-02</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>64</v>
+        <v>137</v>
       </c>
       <c r="F7" t="n">
         <v>4</v>
@@ -807,10 +807,10 @@
         <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -831,7 +831,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EURO_Futures</t>
+          <t>NY_Platinum_Futures</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -842,20 +842,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -867,19 +867,19 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>6.25</v>
+        <v>6.63</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>106253.5</v>
+        <v>106631.02</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>NY_Palladium_Futures</t>
+          <t>EURO_Futures</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -890,11 +890,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -918,31 +918,31 @@
         <v>100</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>6.22</v>
+        <v>6.25</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>106216.17</v>
+        <v>106253.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bitcoin_Per_USD_CME</t>
+          <t>NY_Palladium_Futures</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -966,34 +966,34 @@
         <v>100</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>5.38</v>
+        <v>6.22</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>105381.31</v>
+        <v>106216.17</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Corn_CBOT_Futures</t>
+          <t>Bitcoin_Per_USD_CME</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -1002,22 +1002,22 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>4.62</v>
+        <v>5.38</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>104620.42</v>
+        <v>105381.31</v>
       </c>
     </row>
     <row r="12">
@@ -1034,11 +1034,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -1082,11 +1082,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -1130,11 +1130,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F14" t="n">
         <v>2</v>
@@ -1178,11 +1178,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
@@ -1226,11 +1226,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -1271,11 +1271,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1361,11 +1361,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1406,11 +1406,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1451,11 +1451,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1496,11 +1496,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
@@ -1544,11 +1544,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
@@ -1592,11 +1592,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -1640,11 +1640,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -1688,11 +1688,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-24); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-28 05:43 UTC.</t>
+          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-27); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-28 16:18 UTC.</t>
         </is>
       </c>
     </row>
@@ -3301,6 +3301,14 @@
           <t>2026-07-24</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
       <c r="G13" t="n">
         <v>706</v>
       </c>
@@ -3310,16 +3318,25 @@
       <c r="I13" t="n">
         <v>695.9</v>
       </c>
+      <c r="J13" t="n">
+        <v>695.9</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>open_at_end</t>
-        </is>
+          <t>target_r</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N13" t="n">
         <v>113921.15</v>
       </c>
       <c r="O13" t="n">
-        <v>113921.15</v>
+        <v>116929.81</v>
       </c>
     </row>
     <row r="14">
@@ -3902,6 +3919,14 @@
           <t>2026-07-24</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
       <c r="G24" t="n">
         <v>488.1</v>
       </c>
@@ -3911,16 +3936,25 @@
       <c r="I24" t="n">
         <v>480.5</v>
       </c>
+      <c r="J24" t="n">
+        <v>480.5</v>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>open_at_end</t>
-        </is>
+          <t>target_r</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N24" t="n">
         <v>104620.42</v>
       </c>
       <c r="O24" t="n">
-        <v>104620.42</v>
+        <v>107383.44</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Output churn from the latest pipeline run
A new array day: quickfix goes 90 -> 91 trades, final capital
322,043.71 -> 321,987.76. Regenerated reports, charter hand-off files
and workbooks follow. No rule, fill model or registry change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/quickfix_all_markets_daily.xlsx
+++ b/output/quickfix_all_markets_daily.xlsx
@@ -554,11 +554,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F2" t="n">
         <v>9</v>
@@ -602,11 +602,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F3" t="n">
         <v>6</v>
@@ -650,17 +650,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
@@ -675,13 +675,13 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>66.7</v>
+        <v>70</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>12.92</v>
+        <v>15.9</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>112916.93</v>
+        <v>115899.07</v>
       </c>
     </row>
     <row r="5">
@@ -698,11 +698,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F5" t="n">
         <v>4</v>
@@ -746,11 +746,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -794,11 +794,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F7" t="n">
         <v>4</v>
@@ -842,11 +842,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F8" t="n">
         <v>4</v>
@@ -890,11 +890,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -938,11 +938,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -986,11 +986,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -1034,11 +1034,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -1082,11 +1082,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -1130,11 +1130,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F14" t="n">
         <v>2</v>
@@ -1152,7 +1152,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>50</v>
@@ -1178,11 +1178,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
@@ -1226,11 +1226,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -1271,11 +1271,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1361,11 +1361,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1406,11 +1406,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1451,11 +1451,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1496,11 +1496,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
@@ -1544,11 +1544,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
@@ -1592,11 +1592,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -1640,11 +1640,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -1688,11 +1688,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-27); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-29 02:46 UTC.</t>
+          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-29); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-30 20:33 UTC.</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O91"/>
+  <dimension ref="A1:O93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5778,11 +5778,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NY_Palladium_Futures</t>
+          <t>NY_Natural_Gas_Futures</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -5791,45 +5791,28 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>1</v>
+          <t>2026-07-29</t>
+        </is>
       </c>
       <c r="G57" t="n">
-        <v>1360.4</v>
+        <v>2.69</v>
       </c>
       <c r="H57" t="n">
-        <v>1343.4</v>
+        <v>2.665</v>
       </c>
       <c r="I57" t="n">
-        <v>1392.7</v>
-      </c>
-      <c r="J57" t="n">
-        <v>1403</v>
+        <v>2.737</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>target_r</t>
-        </is>
-      </c>
-      <c r="L57" t="n">
-        <v>2.5059</v>
-      </c>
-      <c r="M57" s="2" t="n">
-        <v>3.4832</v>
+          <t>open_at_end</t>
+        </is>
       </c>
       <c r="N57" t="n">
-        <v>100000</v>
+        <v>101214.29</v>
       </c>
       <c r="O57" t="n">
-        <v>103483.18</v>
+        <v>101214.29</v>
       </c>
     </row>
     <row r="58">
@@ -5839,7 +5822,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -5848,28 +5831,28 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F58" t="n">
         <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>1167</v>
+        <v>1360.4</v>
       </c>
       <c r="H58" t="n">
-        <v>1159.4</v>
+        <v>1343.4</v>
       </c>
       <c r="I58" t="n">
-        <v>1181.4</v>
+        <v>1392.7</v>
       </c>
       <c r="J58" t="n">
-        <v>1181.4</v>
+        <v>1403</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -5877,56 +5860,56 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>1.9</v>
+        <v>2.5059</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>2.641</v>
+        <v>3.4832</v>
       </c>
       <c r="N58" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O58" t="n">
         <v>103483.18</v>
-      </c>
-      <c r="O58" t="n">
-        <v>106216.17</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NY_Platinum_Futures</t>
+          <t>NY_Palladium_Futures</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>2084.6</v>
+        <v>1167</v>
       </c>
       <c r="H59" t="n">
-        <v>2113.7</v>
+        <v>1159.4</v>
       </c>
       <c r="I59" t="n">
-        <v>2029.3</v>
+        <v>1181.4</v>
       </c>
       <c r="J59" t="n">
-        <v>2029.3</v>
+        <v>1181.4</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -5940,10 +5923,10 @@
         <v>2.641</v>
       </c>
       <c r="N59" t="n">
-        <v>100000</v>
+        <v>103483.18</v>
       </c>
       <c r="O59" t="n">
-        <v>102641</v>
+        <v>106216.17</v>
       </c>
     </row>
     <row r="60">
@@ -5953,54 +5936,54 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="F60" t="n">
         <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>1641.5</v>
+        <v>2084.6</v>
       </c>
       <c r="H60" t="n">
-        <v>1621</v>
+        <v>2113.7</v>
       </c>
       <c r="I60" t="n">
-        <v>1680.5</v>
+        <v>2029.3</v>
       </c>
       <c r="J60" t="n">
-        <v>1621</v>
+        <v>2029.3</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L60" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M60" s="5" t="n">
-        <v>-1.39</v>
+        <v>1.9</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N60" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O60" t="n">
         <v>102641</v>
-      </c>
-      <c r="O60" t="n">
-        <v>101214.29</v>
       </c>
     </row>
     <row r="61">
@@ -6010,7 +5993,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -6019,45 +6002,45 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="F61" t="n">
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>1581.5</v>
+        <v>1641.5</v>
       </c>
       <c r="H61" t="n">
-        <v>1547.6</v>
+        <v>1621</v>
       </c>
       <c r="I61" t="n">
-        <v>1645.9</v>
+        <v>1680.5</v>
       </c>
       <c r="J61" t="n">
-        <v>1645.9</v>
+        <v>1621</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L61" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M61" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M61" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N61" t="n">
+        <v>102641</v>
+      </c>
+      <c r="O61" t="n">
         <v>101214.29</v>
-      </c>
-      <c r="O61" t="n">
-        <v>103887.36</v>
       </c>
     </row>
     <row r="62">
@@ -6067,7 +6050,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -6076,28 +6059,28 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>1559</v>
+        <v>1581.5</v>
       </c>
       <c r="H62" t="n">
-        <v>1539.5</v>
+        <v>1547.6</v>
       </c>
       <c r="I62" t="n">
-        <v>1596</v>
+        <v>1645.9</v>
       </c>
       <c r="J62" t="n">
-        <v>1596</v>
+        <v>1645.9</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -6111,70 +6094,73 @@
         <v>2.641</v>
       </c>
       <c r="N62" t="n">
+        <v>101214.29</v>
+      </c>
+      <c r="O62" t="n">
         <v>103887.36</v>
-      </c>
-      <c r="O62" t="n">
-        <v>106631.02</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Nasdaq_100_E_mini</t>
+          <t>NY_Platinum_Futures</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F63" t="n">
         <v>1</v>
       </c>
       <c r="G63" t="n">
-        <v>27907</v>
+        <v>1559</v>
       </c>
       <c r="H63" t="n">
-        <v>27965.76</v>
+        <v>1539.5</v>
       </c>
       <c r="I63" t="n">
-        <v>27795.36</v>
+        <v>1596</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1596</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>unknown_pl</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L63" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M63" s="5" t="n">
-        <v>-1.39</v>
+        <v>1.9</v>
+      </c>
+      <c r="M63" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N63" t="n">
-        <v>100000</v>
+        <v>103887.36</v>
       </c>
       <c r="O63" t="n">
-        <v>98610</v>
+        <v>106631.02</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S_P_500_E_mini</t>
+          <t>Nasdaq_100_E_mini</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -6187,51 +6173,48 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="F64" t="n">
         <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>7206.55</v>
+        <v>27907</v>
       </c>
       <c r="H64" t="n">
-        <v>7223.26</v>
+        <v>27965.76</v>
       </c>
       <c r="I64" t="n">
-        <v>7174.8</v>
-      </c>
-      <c r="J64" t="n">
-        <v>7174.8</v>
+        <v>27795.36</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>unknown_pl</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M64" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M64" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N64" t="n">
         <v>100000</v>
       </c>
       <c r="O64" t="n">
-        <v>102641</v>
+        <v>98610</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S_P_500_Index</t>
+          <t>S_P_500_E_mini</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -6244,28 +6227,28 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="F65" t="n">
         <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>6957.43</v>
+        <v>7206.55</v>
       </c>
       <c r="H65" t="n">
-        <v>6965.7</v>
+        <v>7223.26</v>
       </c>
       <c r="I65" t="n">
-        <v>6941.72</v>
+        <v>7174.8</v>
       </c>
       <c r="J65" t="n">
-        <v>6941.72</v>
+        <v>7174.8</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -6292,7 +6275,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -6301,45 +6284,45 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="F66" t="n">
         <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>6982.4</v>
+        <v>6957.43</v>
       </c>
       <c r="H66" t="n">
-        <v>6988.83</v>
+        <v>6965.7</v>
       </c>
       <c r="I66" t="n">
-        <v>6970.18</v>
+        <v>6941.72</v>
       </c>
       <c r="J66" t="n">
-        <v>7002</v>
+        <v>6941.72</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L66" t="n">
-        <v>-3.0482</v>
-      </c>
-      <c r="M66" s="5" t="n">
-        <v>-4.237</v>
+        <v>1.9</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N66" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O66" t="n">
         <v>102641</v>
-      </c>
-      <c r="O66" t="n">
-        <v>98292.09</v>
       </c>
     </row>
     <row r="67">
@@ -6349,7 +6332,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -6358,12 +6341,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -6373,30 +6356,30 @@
         <v>6982.4</v>
       </c>
       <c r="H67" t="n">
-        <v>6992.85</v>
+        <v>6988.83</v>
       </c>
       <c r="I67" t="n">
-        <v>6962.54</v>
+        <v>6970.18</v>
       </c>
       <c r="J67" t="n">
-        <v>6947.27</v>
+        <v>7002</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L67" t="n">
-        <v>3.3617</v>
-      </c>
-      <c r="M67" s="2" t="n">
-        <v>4.6728</v>
+        <v>-3.0482</v>
+      </c>
+      <c r="M67" s="5" t="n">
+        <v>-4.237</v>
       </c>
       <c r="N67" t="n">
+        <v>102641</v>
+      </c>
+      <c r="O67" t="n">
         <v>98292.09</v>
-      </c>
-      <c r="O67" t="n">
-        <v>102885.07</v>
       </c>
     </row>
     <row r="68">
@@ -6406,7 +6389,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -6415,12 +6398,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -6430,27 +6413,30 @@
         <v>6982.4</v>
       </c>
       <c r="H68" t="n">
-        <v>6991.93</v>
+        <v>6992.85</v>
       </c>
       <c r="I68" t="n">
-        <v>6964.29</v>
+        <v>6962.54</v>
+      </c>
+      <c r="J68" t="n">
+        <v>6947.27</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>unknown_pl</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L68" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M68" s="5" t="n">
-        <v>-1.39</v>
+        <v>3.3617</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>4.6728</v>
       </c>
       <c r="N68" t="n">
+        <v>98292.09</v>
+      </c>
+      <c r="O68" t="n">
         <v>102885.07</v>
-      </c>
-      <c r="O68" t="n">
-        <v>101454.97</v>
       </c>
     </row>
     <row r="69">
@@ -6460,7 +6446,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -6469,12 +6455,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -6484,10 +6470,10 @@
         <v>6982.4</v>
       </c>
       <c r="H69" t="n">
-        <v>6986.84</v>
+        <v>6991.93</v>
       </c>
       <c r="I69" t="n">
-        <v>6973.96</v>
+        <v>6964.29</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -6501,10 +6487,10 @@
         <v>-1.39</v>
       </c>
       <c r="N69" t="n">
+        <v>102885.07</v>
+      </c>
+      <c r="O69" t="n">
         <v>101454.97</v>
-      </c>
-      <c r="O69" t="n">
-        <v>100044.75</v>
       </c>
     </row>
     <row r="70">
@@ -6514,94 +6500,91 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="F70" t="n">
         <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>6794.4</v>
+        <v>6982.4</v>
       </c>
       <c r="H70" t="n">
-        <v>6770.77</v>
+        <v>6986.84</v>
       </c>
       <c r="I70" t="n">
-        <v>6839.3</v>
-      </c>
-      <c r="J70" t="n">
-        <v>6769.03</v>
+        <v>6973.96</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>unknown_pl</t>
         </is>
       </c>
       <c r="L70" t="n">
-        <v>-1.0736</v>
+        <v>-1</v>
       </c>
       <c r="M70" s="5" t="n">
-        <v>-1.4924</v>
+        <v>-1.39</v>
       </c>
       <c r="N70" t="n">
+        <v>101454.97</v>
+      </c>
+      <c r="O70" t="n">
         <v>100044.75</v>
-      </c>
-      <c r="O70" t="n">
-        <v>98551.73</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Silver_Futures_COMEX</t>
+          <t>S_P_500_Index</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="F71" t="n">
         <v>1</v>
       </c>
       <c r="G71" t="n">
-        <v>86.081</v>
+        <v>6794.4</v>
       </c>
       <c r="H71" t="n">
-        <v>88.001</v>
+        <v>6770.77</v>
       </c>
       <c r="I71" t="n">
-        <v>82.43300000000001</v>
+        <v>6839.3</v>
       </c>
       <c r="J71" t="n">
-        <v>88.001</v>
+        <v>6769.03</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -6609,16 +6592,16 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>-1</v>
+        <v>-1.0736</v>
       </c>
       <c r="M71" s="5" t="n">
-        <v>-1.39</v>
+        <v>-1.4924</v>
       </c>
       <c r="N71" t="n">
-        <v>100000</v>
+        <v>100044.75</v>
       </c>
       <c r="O71" t="n">
-        <v>98610</v>
+        <v>98551.73</v>
       </c>
     </row>
     <row r="72">
@@ -6628,117 +6611,117 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G72" t="n">
-        <v>73.84399999999999</v>
+        <v>86.081</v>
       </c>
       <c r="H72" t="n">
-        <v>71.999</v>
+        <v>88.001</v>
       </c>
       <c r="I72" t="n">
-        <v>77.349</v>
+        <v>82.43300000000001</v>
       </c>
       <c r="J72" t="n">
-        <v>77.349</v>
+        <v>88.001</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L72" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M72" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M72" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N72" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O72" t="n">
         <v>98610</v>
-      </c>
-      <c r="O72" t="n">
-        <v>101214.29</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Sugar_World_CSCE_Futures</t>
+          <t>Silver_Futures_COMEX</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F73" t="n">
         <v>2</v>
       </c>
       <c r="G73" t="n">
-        <v>15</v>
+        <v>73.84399999999999</v>
       </c>
       <c r="H73" t="n">
-        <v>15.26</v>
+        <v>71.999</v>
       </c>
       <c r="I73" t="n">
-        <v>14.51</v>
+        <v>77.349</v>
       </c>
       <c r="J73" t="n">
-        <v>15.26</v>
+        <v>77.349</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L73" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M73" s="5" t="n">
-        <v>-1.39</v>
+        <v>1.9</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N73" t="n">
-        <v>100000</v>
+        <v>98610</v>
       </c>
       <c r="O73" t="n">
-        <v>98610</v>
+        <v>101214.29</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Teucrium_Wheat_Fund</t>
+          <t>Sugar_World_CSCE_Futures</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -6751,28 +6734,28 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G74" t="n">
-        <v>20.89</v>
+        <v>15</v>
       </c>
       <c r="H74" t="n">
-        <v>21.07</v>
+        <v>15.26</v>
       </c>
       <c r="I74" t="n">
-        <v>20.55</v>
+        <v>14.51</v>
       </c>
       <c r="J74" t="n">
-        <v>21.08</v>
+        <v>15.26</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -6780,22 +6763,22 @@
         </is>
       </c>
       <c r="L74" t="n">
-        <v>-1.0556</v>
+        <v>-1</v>
       </c>
       <c r="M74" s="5" t="n">
-        <v>-1.4672</v>
+        <v>-1.39</v>
       </c>
       <c r="N74" t="n">
         <v>100000</v>
       </c>
       <c r="O74" t="n">
-        <v>98532.78</v>
+        <v>98610</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>USD_EUR_Cross_Rate</t>
+          <t>Teucrium_Wheat_Fund</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -6808,28 +6791,28 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="F75" t="n">
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>0.8614000000000001</v>
+        <v>20.89</v>
       </c>
       <c r="H75" t="n">
-        <v>0.8637</v>
+        <v>21.07</v>
       </c>
       <c r="I75" t="n">
-        <v>0.857</v>
+        <v>20.55</v>
       </c>
       <c r="J75" t="n">
-        <v>0.8637</v>
+        <v>21.08</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -6837,16 +6820,16 @@
         </is>
       </c>
       <c r="L75" t="n">
-        <v>-1</v>
+        <v>-1.0556</v>
       </c>
       <c r="M75" s="5" t="n">
-        <v>-1.39</v>
+        <v>-1.4672</v>
       </c>
       <c r="N75" t="n">
         <v>100000</v>
       </c>
       <c r="O75" t="n">
-        <v>98610</v>
+        <v>98532.78</v>
       </c>
     </row>
     <row r="76">
@@ -6856,7 +6839,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -6865,12 +6848,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -6880,13 +6863,13 @@
         <v>0.8614000000000001</v>
       </c>
       <c r="H76" t="n">
-        <v>0.8658</v>
+        <v>0.8637</v>
       </c>
       <c r="I76" t="n">
-        <v>0.853</v>
+        <v>0.857</v>
       </c>
       <c r="J76" t="n">
-        <v>0.8658</v>
+        <v>0.8637</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -6900,10 +6883,10 @@
         <v>-1.39</v>
       </c>
       <c r="N76" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O76" t="n">
         <v>98610</v>
-      </c>
-      <c r="O76" t="n">
-        <v>97239.32000000001</v>
       </c>
     </row>
     <row r="77">
@@ -6913,111 +6896,111 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>0.8467</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="H77" t="n">
-        <v>0.8436</v>
+        <v>0.8658</v>
       </c>
       <c r="I77" t="n">
-        <v>0.8526</v>
+        <v>0.853</v>
       </c>
       <c r="J77" t="n">
-        <v>0.8498</v>
+        <v>0.8658</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>data_end</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L77" t="n">
-        <v>1</v>
-      </c>
-      <c r="M77" s="2" t="n">
-        <v>1.39</v>
+        <v>-1</v>
+      </c>
+      <c r="M77" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N77" t="n">
+        <v>98610</v>
+      </c>
+      <c r="O77" t="n">
         <v>97239.32000000001</v>
-      </c>
-      <c r="O77" t="n">
-        <v>98590.95</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>US_30_Year_T_Bond_Futures_CBOT</t>
+          <t>USD_EUR_Cross_Rate</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="F78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>116.5</v>
+        <v>0.8467</v>
       </c>
       <c r="H78" t="n">
-        <v>116.79</v>
+        <v>0.8436</v>
       </c>
       <c r="I78" t="n">
-        <v>115.95</v>
+        <v>0.8526</v>
       </c>
       <c r="J78" t="n">
-        <v>116.79</v>
+        <v>0.8498</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>data_end</t>
         </is>
       </c>
       <c r="L78" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M78" s="5" t="n">
-        <v>-1.39</v>
+        <v>1</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>1.39</v>
       </c>
       <c r="N78" t="n">
-        <v>100000</v>
+        <v>97239.32000000001</v>
       </c>
       <c r="O78" t="n">
-        <v>98610</v>
+        <v>98590.95</v>
       </c>
     </row>
     <row r="79">
@@ -7027,7 +7010,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -7036,45 +7019,45 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="F79" t="n">
         <v>1</v>
       </c>
       <c r="G79" t="n">
-        <v>118.02</v>
+        <v>116.5</v>
       </c>
       <c r="H79" t="n">
-        <v>118.16</v>
+        <v>116.79</v>
       </c>
       <c r="I79" t="n">
-        <v>117.75</v>
+        <v>115.95</v>
       </c>
       <c r="J79" t="n">
-        <v>117.75</v>
+        <v>116.79</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L79" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M79" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M79" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N79" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O79" t="n">
         <v>98610</v>
-      </c>
-      <c r="O79" t="n">
-        <v>101214.29</v>
       </c>
     </row>
     <row r="80">
@@ -7084,7 +7067,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -7093,99 +7076,99 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>1</v>
       </c>
       <c r="G80" t="n">
-        <v>118.08</v>
+        <v>118.02</v>
       </c>
       <c r="H80" t="n">
         <v>118.16</v>
       </c>
       <c r="I80" t="n">
-        <v>117.93</v>
+        <v>117.75</v>
+      </c>
+      <c r="J80" t="n">
+        <v>117.75</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>unknown_pl</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M80" s="5" t="n">
-        <v>-1.39</v>
+        <v>1.9</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N80" t="n">
+        <v>98610</v>
+      </c>
+      <c r="O80" t="n">
         <v>101214.29</v>
-      </c>
-      <c r="O80" t="n">
-        <v>99807.41</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>US_Dollar_Index_Futures</t>
+          <t>US_30_Year_T_Bond_Futures_CBOT</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="F81" t="n">
         <v>1</v>
       </c>
       <c r="G81" t="n">
-        <v>97.81399999999999</v>
+        <v>118.08</v>
       </c>
       <c r="H81" t="n">
-        <v>97.569</v>
+        <v>118.16</v>
       </c>
       <c r="I81" t="n">
-        <v>98.279</v>
-      </c>
-      <c r="J81" t="n">
-        <v>98.279</v>
+        <v>117.93</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>unknown_pl</t>
         </is>
       </c>
       <c r="L81" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M81" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M81" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N81" t="n">
-        <v>100000</v>
+        <v>101214.29</v>
       </c>
       <c r="O81" t="n">
-        <v>102641</v>
+        <v>99807.41</v>
       </c>
     </row>
     <row r="82">
@@ -7195,7 +7178,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -7204,28 +7187,28 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>97.714</v>
+        <v>97.81399999999999</v>
       </c>
       <c r="H82" t="n">
-        <v>97.46899999999999</v>
+        <v>97.569</v>
       </c>
       <c r="I82" t="n">
-        <v>98.18000000000001</v>
+        <v>98.279</v>
       </c>
       <c r="J82" t="n">
-        <v>98.18000000000001</v>
+        <v>98.279</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -7239,10 +7222,10 @@
         <v>2.641</v>
       </c>
       <c r="N82" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O82" t="n">
         <v>102641</v>
-      </c>
-      <c r="O82" t="n">
-        <v>105351.75</v>
       </c>
     </row>
     <row r="83">
@@ -7252,37 +7235,37 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G83" t="n">
-        <v>99.376</v>
+        <v>97.714</v>
       </c>
       <c r="H83" t="n">
-        <v>99.571</v>
+        <v>97.46899999999999</v>
       </c>
       <c r="I83" t="n">
-        <v>99.006</v>
+        <v>98.18000000000001</v>
       </c>
       <c r="J83" t="n">
-        <v>99.006</v>
+        <v>98.18000000000001</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -7296,10 +7279,10 @@
         <v>2.641</v>
       </c>
       <c r="N83" t="n">
+        <v>102641</v>
+      </c>
+      <c r="O83" t="n">
         <v>105351.75</v>
-      </c>
-      <c r="O83" t="n">
-        <v>108134.09</v>
       </c>
     </row>
     <row r="84">
@@ -7309,7 +7292,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -7318,45 +7301,45 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="F84" t="n">
         <v>3</v>
       </c>
       <c r="G84" t="n">
-        <v>99.246</v>
+        <v>99.376</v>
       </c>
       <c r="H84" t="n">
-        <v>99.501</v>
+        <v>99.571</v>
       </c>
       <c r="I84" t="n">
-        <v>98.761</v>
+        <v>99.006</v>
       </c>
       <c r="J84" t="n">
-        <v>99.501</v>
+        <v>99.006</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L84" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M84" s="5" t="n">
-        <v>-1.39</v>
+        <v>1.9</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N84" t="n">
+        <v>105351.75</v>
+      </c>
+      <c r="O84" t="n">
         <v>108134.09</v>
-      </c>
-      <c r="O84" t="n">
-        <v>106631.02</v>
       </c>
     </row>
     <row r="85">
@@ -7366,7 +7349,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -7375,45 +7358,45 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="F85" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G85" t="n">
-        <v>100.066</v>
+        <v>99.246</v>
       </c>
       <c r="H85" t="n">
-        <v>100.201</v>
+        <v>99.501</v>
       </c>
       <c r="I85" t="n">
-        <v>99.809</v>
+        <v>98.761</v>
       </c>
       <c r="J85" t="n">
-        <v>99.809</v>
+        <v>99.501</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L85" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M85" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M85" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N85" t="n">
+        <v>108134.09</v>
+      </c>
+      <c r="O85" t="n">
         <v>106631.02</v>
-      </c>
-      <c r="O85" t="n">
-        <v>109447.15</v>
       </c>
     </row>
     <row r="86">
@@ -7423,7 +7406,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -7432,12 +7415,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F86" t="n">
@@ -7447,13 +7430,13 @@
         <v>100.066</v>
       </c>
       <c r="H86" t="n">
-        <v>100.316</v>
+        <v>100.201</v>
       </c>
       <c r="I86" t="n">
-        <v>99.59099999999999</v>
+        <v>99.809</v>
       </c>
       <c r="J86" t="n">
-        <v>99.45999999999999</v>
+        <v>99.809</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -7461,16 +7444,16 @@
         </is>
       </c>
       <c r="L86" t="n">
-        <v>2.424</v>
+        <v>1.9</v>
       </c>
       <c r="M86" s="2" t="n">
-        <v>3.3694</v>
+        <v>2.641</v>
       </c>
       <c r="N86" t="n">
+        <v>106631.02</v>
+      </c>
+      <c r="O86" t="n">
         <v>109447.15</v>
-      </c>
-      <c r="O86" t="n">
-        <v>113134.82</v>
       </c>
     </row>
     <row r="87">
@@ -7480,7 +7463,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -7489,12 +7472,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -7504,30 +7487,30 @@
         <v>100.066</v>
       </c>
       <c r="H87" t="n">
-        <v>100.361</v>
+        <v>100.316</v>
       </c>
       <c r="I87" t="n">
-        <v>99.505</v>
+        <v>99.59099999999999</v>
       </c>
       <c r="J87" t="n">
-        <v>100.361</v>
+        <v>99.45999999999999</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>target_r</t>
         </is>
       </c>
       <c r="L87" t="n">
-        <v>-1</v>
-      </c>
-      <c r="M87" s="5" t="n">
-        <v>-1.39</v>
+        <v>2.424</v>
+      </c>
+      <c r="M87" s="2" t="n">
+        <v>3.3694</v>
       </c>
       <c r="N87" t="n">
+        <v>109447.15</v>
+      </c>
+      <c r="O87" t="n">
         <v>113134.82</v>
-      </c>
-      <c r="O87" t="n">
-        <v>111562.24</v>
       </c>
     </row>
     <row r="88">
@@ -7537,7 +7520,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -7546,28 +7529,28 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G88" t="n">
-        <v>100.621</v>
+        <v>100.066</v>
       </c>
       <c r="H88" t="n">
-        <v>100.911</v>
+        <v>100.361</v>
       </c>
       <c r="I88" t="n">
-        <v>100.07</v>
+        <v>99.505</v>
       </c>
       <c r="J88" t="n">
-        <v>100.911</v>
+        <v>100.361</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -7581,10 +7564,10 @@
         <v>-1.39</v>
       </c>
       <c r="N88" t="n">
+        <v>113134.82</v>
+      </c>
+      <c r="O88" t="n">
         <v>111562.24</v>
-      </c>
-      <c r="O88" t="n">
-        <v>110011.53</v>
       </c>
     </row>
     <row r="89">
@@ -7594,7 +7577,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -7603,55 +7586,55 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G89" t="n">
-        <v>101.411</v>
+        <v>100.621</v>
       </c>
       <c r="H89" t="n">
-        <v>101.526</v>
+        <v>100.911</v>
       </c>
       <c r="I89" t="n">
-        <v>101.192</v>
+        <v>100.07</v>
       </c>
       <c r="J89" t="n">
-        <v>101.192</v>
+        <v>100.911</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>target_r</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="L89" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="M89" s="2" t="n">
-        <v>2.641</v>
+        <v>-1</v>
+      </c>
+      <c r="M89" s="5" t="n">
+        <v>-1.39</v>
       </c>
       <c r="N89" t="n">
+        <v>111562.24</v>
+      </c>
+      <c r="O89" t="n">
         <v>110011.53</v>
-      </c>
-      <c r="O89" t="n">
-        <v>112916.93</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>United_States_Oil_Fund_LP</t>
+          <t>US_Dollar_Index_Futures</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -7660,28 +7643,28 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F90" t="n">
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>121.72</v>
+        <v>101.411</v>
       </c>
       <c r="H90" t="n">
-        <v>123.03</v>
+        <v>101.526</v>
       </c>
       <c r="I90" t="n">
-        <v>119.23</v>
+        <v>101.192</v>
       </c>
       <c r="J90" t="n">
-        <v>113.29</v>
+        <v>101.192</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -7689,26 +7672,26 @@
         </is>
       </c>
       <c r="L90" t="n">
-        <v>6.4351</v>
+        <v>1.9</v>
       </c>
       <c r="M90" s="2" t="n">
-        <v>8.944800000000001</v>
+        <v>2.641</v>
       </c>
       <c r="N90" t="n">
-        <v>100000</v>
+        <v>110011.53</v>
       </c>
       <c r="O90" t="n">
-        <v>108944.81</v>
+        <v>112916.93</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>United_States_Oil_Fund_LP</t>
+          <t>US_Dollar_Index_Futures</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -7717,28 +7700,28 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F91" t="n">
         <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>130.16</v>
+        <v>101.411</v>
       </c>
       <c r="H91" t="n">
-        <v>130.94</v>
+        <v>101.491</v>
       </c>
       <c r="I91" t="n">
-        <v>128.68</v>
+        <v>101.259</v>
       </c>
       <c r="J91" t="n">
-        <v>128.68</v>
+        <v>101.259</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -7752,9 +7735,123 @@
         <v>2.641</v>
       </c>
       <c r="N91" t="n">
+        <v>112916.93</v>
+      </c>
+      <c r="O91" t="n">
+        <v>115899.07</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>United_States_Oil_Fund_LP</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" t="n">
+        <v>121.72</v>
+      </c>
+      <c r="H92" t="n">
+        <v>123.03</v>
+      </c>
+      <c r="I92" t="n">
+        <v>119.23</v>
+      </c>
+      <c r="J92" t="n">
+        <v>113.29</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>target_r</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>6.4351</v>
+      </c>
+      <c r="M92" s="2" t="n">
+        <v>8.944800000000001</v>
+      </c>
+      <c r="N92" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O92" t="n">
         <v>108944.81</v>
       </c>
-      <c r="O91" t="n">
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>United_States_Oil_Fund_LP</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" t="n">
+        <v>130.16</v>
+      </c>
+      <c r="H93" t="n">
+        <v>130.94</v>
+      </c>
+      <c r="I93" t="n">
+        <v>128.68</v>
+      </c>
+      <c r="J93" t="n">
+        <v>128.68</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>target_r</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M93" s="2" t="n">
+        <v>2.641</v>
+      </c>
+      <c r="N93" t="n">
+        <v>108944.81</v>
+      </c>
+      <c r="O93" t="n">
         <v>111822.04</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Three more bar exits, and the stop that comes with them
Rule 4's bar exits become a family parameterised by WHICH BAR the trade is
marked out on, counting the entry bar as bar 0. quickfixopen becomes
quickfixopen1, and quickfixclose1, quickfixopen2 and quickfixclose2 join it.

The stop is not rule 4, so a bar exit held past its entry bar keeps it: on
every bar in between it is resolved by the same check_exit, handed a policy
that never has a target. On the exit bar an open exit wins outright (nothing
trades ahead of a bar's first price) and a close exit yields to the stop (a
stop triggers intraday, a market-on-close at the bell). Rule4.bar_exit_at is
which, and it is required beside a bar_exit.

No new exit reason: exit_close and exit_open name the order type, not the bar,
so all five share them and charter needs no change beyond its docs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/quickfix_all_markets_daily.xlsx
+++ b/output/quickfix_all_markets_daily.xlsx
@@ -554,11 +554,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F2" t="n">
         <v>9</v>
@@ -602,11 +602,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" t="n">
         <v>6</v>
@@ -650,11 +650,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
@@ -698,11 +698,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F5" t="n">
         <v>4</v>
@@ -746,11 +746,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -794,11 +794,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F7" t="n">
         <v>4</v>
@@ -842,11 +842,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F8" t="n">
         <v>4</v>
@@ -890,11 +890,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -938,11 +938,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -986,11 +986,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -1023,7 +1023,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>German_Long_Bund</t>
+          <t>NY_Natural_Gas_Futures</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1034,20 +1034,20 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -1059,34 +1059,34 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>2.64</v>
+        <v>3.89</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>102641</v>
+        <v>103887.36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S_P_500_E_mini</t>
+          <t>German_Long_Bund</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -1119,31 +1119,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>NY_Natural_Gas_Futures</t>
+          <t>S_P_500_E_mini</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1152,16 +1152,16 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1.21</v>
+        <v>2.64</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>101214.29</v>
+        <v>102641</v>
       </c>
     </row>
     <row r="15">
@@ -1178,11 +1178,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
@@ -1226,11 +1226,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -1271,11 +1271,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1361,11 +1361,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1406,11 +1406,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1451,11 +1451,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1496,11 +1496,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
@@ -1544,11 +1544,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
@@ -1592,11 +1592,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -1640,11 +1640,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -1688,11 +1688,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-29); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-30 20:33 UTC.</t>
+          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-30); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-31 15:45 UTC.</t>
         </is>
       </c>
     </row>
@@ -5794,6 +5794,14 @@
           <t>2026-07-29</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
       <c r="G57" t="n">
         <v>2.69</v>
       </c>
@@ -5803,16 +5811,25 @@
       <c r="I57" t="n">
         <v>2.737</v>
       </c>
+      <c r="J57" t="n">
+        <v>2.737</v>
+      </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>open_at_end</t>
-        </is>
+          <t>target_r</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M57" s="2" t="n">
+        <v>2.641</v>
       </c>
       <c r="N57" t="n">
         <v>101214.29</v>
       </c>
       <c r="O57" t="n">
-        <v>101214.29</v>
+        <v>103887.36</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
Output churn from a fresh array day
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/quickfix_all_markets_daily.xlsx
+++ b/output/quickfix_all_markets_daily.xlsx
@@ -554,11 +554,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F2" t="n">
         <v>9</v>
@@ -602,11 +602,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F3" t="n">
         <v>6</v>
@@ -650,11 +650,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
@@ -698,11 +698,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F5" t="n">
         <v>4</v>
@@ -746,11 +746,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -794,11 +794,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F7" t="n">
         <v>4</v>
@@ -842,11 +842,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F8" t="n">
         <v>4</v>
@@ -890,11 +890,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -938,11 +938,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -986,11 +986,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -1034,11 +1034,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
@@ -1082,11 +1082,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -1130,11 +1130,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
@@ -1178,11 +1178,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
@@ -1226,11 +1226,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -1271,11 +1271,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1361,11 +1361,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1406,11 +1406,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1451,11 +1451,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1496,11 +1496,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
@@ -1544,11 +1544,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
@@ -1592,11 +1592,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -1640,11 +1640,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -1688,11 +1688,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-30); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-07-31 17:02 UTC.</t>
+          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-31); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-08-01 19:43 UTC.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
quickfix1m1dc v2: market-order entries, ladder stops, two dials, 2x2 run
Lode's audit decisions implemented. Entry is a market order the moment
the first reversal PRINTS (or is gapped past - then fill from the open),
4 ticks adverse slippage, R denominated level-to-stop; stop one tick
beyond the 5th reversal (4th when only four; ladder must carry four);
tightening and the overnight window became dials. Mondays trade from the
open in blocked mode - the Saturday landing IS Monday's update. Two bugs
the first matrix pass caught: ICE sentinel prices leaking into bar opens
(all four OHLC fields now sanitized) and a touch-trigger that fired with
price merely beyond the level. 15 synthetic tests rewritten and green.
run_1m_matrix.py runs the 2x2 in one data pass: frozen+blocked leads on
every priority metric (130 trades, wr 30.8, +19.25R, streak 7, DD 23.3%).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/quickfix_all_markets_daily.xlsx
+++ b/output/quickfix_all_markets_daily.xlsx
@@ -554,11 +554,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F2" t="n">
         <v>9</v>
@@ -602,11 +602,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F3" t="n">
         <v>6</v>
@@ -650,11 +650,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
@@ -698,11 +698,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" t="n">
         <v>4</v>
@@ -746,11 +746,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -794,11 +794,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F7" t="n">
         <v>4</v>
@@ -842,11 +842,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F8" t="n">
         <v>4</v>
@@ -890,11 +890,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F9" t="n">
         <v>2</v>
@@ -938,11 +938,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -986,11 +986,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F11" t="n">
         <v>2</v>
@@ -1034,11 +1034,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
@@ -1082,11 +1082,11 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -1130,11 +1130,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
@@ -1178,11 +1178,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F15" t="n">
         <v>2</v>
@@ -1226,11 +1226,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -1271,11 +1271,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1316,11 +1316,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1361,11 +1361,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1406,11 +1406,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1451,11 +1451,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1496,11 +1496,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F22" t="n">
         <v>3</v>
@@ -1544,11 +1544,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
@@ -1592,11 +1592,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
@@ -1640,11 +1640,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -1688,11 +1688,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-07-31); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-08-02 00:09 UTC.</t>
+          <t>quickfix daily (target = 1.9R, or an opposite reversal nearer than 1.9R), starting capital 100,000, risk 1.39%/trade, fees 0.0. obsolete = last bar &gt; 30d before newest (2026-08-04); a position still open on an obsolete market's last bar is flattened at that bar's close (data_end). generated 2026-08-05 13:32 UTC.</t>
         </is>
       </c>
     </row>

</xml_diff>